<commit_message>
misc: continuing with project setup
</commit_message>
<xml_diff>
--- a/docs/worklog.xlsx
+++ b/docs/worklog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Trimestre3\PreTPI\DocFlow\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383A6786-81B2-4858-B97B-84FF988F5FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E52A7AD-4694-49F6-B5E1-BBA662B48828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E47AB7C-07D2-4047-9F3F-A43FBD3CD553}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>date</t>
   </si>
@@ -540,18 +540,30 @@
       <c r="D3" s="4">
         <v>0.37847222222222221</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="E3" s="4">
+        <v>0.44791666666666669</v>
+      </c>
       <c r="F3" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+    <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>46056</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>

</xml_diff>

<commit_message>
feat: added first basic UI elements to electron page
</commit_message>
<xml_diff>
--- a/docs/worklog.xlsx
+++ b/docs/worklog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Trimestre3\PreTPI\DocFlow\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E52A7AD-4694-49F6-B5E1-BBA662B48828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4FD2CE-DFE8-44FC-9EAC-693AF87983AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E47AB7C-07D2-4047-9F3F-A43FBD3CD553}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t>date</t>
   </si>
@@ -66,6 +66,15 @@
   </si>
   <si>
     <t>révision du cahier des charges, création du Github Project, familiarisation avec les technos</t>
+  </si>
+  <si>
+    <t>done</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>première feature basique, création des premiers éléments UI de ma fenêtre electron</t>
   </si>
 </sst>
 </file>
@@ -560,18 +569,30 @@
       <c r="D4" s="4">
         <v>0.55555555555555558</v>
       </c>
-      <c r="E4" s="4"/>
+      <c r="E4" s="4">
+        <v>0.59375</v>
+      </c>
       <c r="F4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>46056</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0.59375</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>

</xml_diff>